<commit_message>
Working version of restart broken
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/accelerated_spinup/accelerated_spinup.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/accelerated_spinup/accelerated_spinup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\accelerated_spinup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F9CEDD-A830-4E15-8729-F4B4D9BE1DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6EC517F-7A45-4C10-B4A3-2EACFE1DAA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4188" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="264">
   <si>
     <t>-------------------</t>
   </si>
@@ -819,6 +819,15 @@
   </si>
   <si>
     <t>D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\forcing\Forcing_Data\</t>
+  </si>
+  <si>
+    <t>not necessary unless user wants an output, but could be OUT_do_nothing instead</t>
+  </si>
+  <si>
+    <t>OUT_last_timestep</t>
+  </si>
+  <si>
+    <t>save_timestep</t>
   </si>
 </sst>
 </file>
@@ -1209,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N404"/>
+  <dimension ref="A1:N410"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.54296875" customWidth="1"/>
@@ -1531,6 +1540,9 @@
       <c r="D36" t="s">
         <v>5</v>
       </c>
+      <c r="E36" s="4" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
@@ -2120,7 +2132,10 @@
       <c r="E100" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="F100" s="3" t="s">
+      <c r="F100" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G100" s="3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2140,7 +2155,10 @@
       <c r="E101" s="5">
         <v>1</v>
       </c>
-      <c r="F101" s="3" t="s">
+      <c r="F101" s="5">
+        <v>1</v>
+      </c>
+      <c r="G101" s="3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -3555,1383 +3573,1413 @@
       </c>
     </row>
     <row r="256" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.35"/>
+    <row r="257" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35"/>
     <row r="258" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A258" t="s">
-        <v>0</v>
+      <c r="A258" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B258" s="5" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A259" t="s">
-        <v>98</v>
-      </c>
-      <c r="B259" t="s">
-        <v>2</v>
+      <c r="A259" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="B259" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
+        <v>263</v>
+      </c>
+      <c r="B260" s="5"/>
+    </row>
+    <row r="261" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A261" t="s">
+        <v>8</v>
+      </c>
+      <c r="B261" s="5"/>
+    </row>
+    <row r="262" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35"/>
+    <row r="264" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A264" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A265" t="s">
+        <v>98</v>
+      </c>
+      <c r="B265" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="266" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A266" t="s">
         <v>22</v>
       </c>
-      <c r="B260">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A262" t="s">
+      <c r="B266">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="268" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A268" t="s">
         <v>99</v>
       </c>
-      <c r="B262" t="s">
+      <c r="B268" t="s">
         <v>100</v>
       </c>
-      <c r="C262" t="s">
+      <c r="C268" t="s">
         <v>101</v>
       </c>
-      <c r="D262" t="s">
+      <c r="D268" t="s">
         <v>102</v>
       </c>
-      <c r="E262" t="s">
+      <c r="E268" t="s">
         <v>103</v>
       </c>
-      <c r="F262" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C263">
+      <c r="F268" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="269" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C269">
         <v>0</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D269" s="1">
         <v>0.05</v>
       </c>
-      <c r="E263">
+      <c r="E269">
         <v>0.5</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C264">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C270">
         <v>0.5</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D270" s="1">
         <v>0.05</v>
       </c>
-      <c r="E264">
+      <c r="E270">
         <v>3</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C265">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C271">
         <v>3</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D271" s="1">
         <v>0.1</v>
       </c>
-      <c r="E265">
+      <c r="E271">
         <v>10</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C266">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C272">
         <v>10</v>
       </c>
-      <c r="D266">
-        <v>1</v>
-      </c>
-      <c r="E266">
+      <c r="D272">
+        <v>1</v>
+      </c>
+      <c r="E272">
         <v>50</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C267">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C273">
         <v>50</v>
       </c>
-      <c r="D267" s="1">
-        <v>5</v>
-      </c>
-      <c r="E267">
+      <c r="D273" s="1">
+        <v>5</v>
+      </c>
+      <c r="E273">
         <v>100</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B268" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A269" t="s">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B274" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="275" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A275" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A272" t="s">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A278" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A273" t="s">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A279" t="s">
         <v>104</v>
       </c>
-      <c r="B273" t="s">
+      <c r="B279" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A274" t="s">
-        <v>27</v>
-      </c>
-      <c r="B274">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A276" t="s">
-        <v>105</v>
-      </c>
-      <c r="B276" t="s">
-        <v>106</v>
-      </c>
-      <c r="C276" t="s">
-        <v>107</v>
-      </c>
-      <c r="D276" t="s">
-        <v>108</v>
-      </c>
-      <c r="E276" t="s">
-        <v>5</v>
-      </c>
-      <c r="F276" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B277">
-        <v>0</v>
-      </c>
-      <c r="C277" t="s">
-        <v>124</v>
-      </c>
-      <c r="D277">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B278">
-        <v>5</v>
-      </c>
-      <c r="C278" t="s">
-        <v>156</v>
-      </c>
-      <c r="D278">
-        <v>1</v>
-      </c>
-      <c r="F278" s="4" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B279" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="280" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>110</v>
-      </c>
-      <c r="B280" t="s">
-        <v>160</v>
-      </c>
-      <c r="D280" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A281" t="s">
-        <v>112</v>
-      </c>
-      <c r="B281">
+        <v>27</v>
+      </c>
+      <c r="B280">
         <v>1</v>
       </c>
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B282" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="C282" t="s">
-        <v>5</v>
-      </c>
-      <c r="D282" s="4" t="s">
-        <v>114</v>
+        <v>107</v>
+      </c>
+      <c r="D282" t="s">
+        <v>108</v>
+      </c>
+      <c r="E282" t="s">
+        <v>5</v>
+      </c>
+      <c r="F282" s="4" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="283" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A283" t="s">
-        <v>115</v>
-      </c>
-      <c r="B283" t="s">
-        <v>4</v>
+      <c r="B283">
+        <v>0</v>
       </c>
       <c r="C283" t="s">
-        <v>5</v>
+        <v>124</v>
+      </c>
+      <c r="D283">
+        <v>1</v>
       </c>
     </row>
     <row r="284" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A284" t="s">
-        <v>8</v>
+      <c r="B284">
+        <v>5</v>
+      </c>
+      <c r="C284" t="s">
+        <v>156</v>
+      </c>
+      <c r="D284">
+        <v>1</v>
+      </c>
+      <c r="F284" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="285" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B285" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="286" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A286" t="s">
+        <v>110</v>
+      </c>
+      <c r="B286" t="s">
+        <v>160</v>
+      </c>
+      <c r="D286" s="4" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>0</v>
+        <v>112</v>
+      </c>
+      <c r="B287">
+        <v>1</v>
       </c>
     </row>
     <row r="288" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B288" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="C288" t="s">
+        <v>5</v>
+      </c>
+      <c r="D288" s="4" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
+        <v>115</v>
+      </c>
+      <c r="B289" t="s">
+        <v>4</v>
+      </c>
+      <c r="C289" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="290" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A290" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="293" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A293" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A294" t="s">
+        <v>116</v>
+      </c>
+      <c r="B294" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="295" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A295" t="s">
         <v>30</v>
       </c>
-      <c r="B289">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A291" t="s">
+      <c r="B295">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A297" t="s">
         <v>117</v>
       </c>
-      <c r="B291" t="s">
+      <c r="B297" t="s">
         <v>106</v>
       </c>
-      <c r="C291" t="s">
+      <c r="C297" t="s">
         <v>118</v>
       </c>
-      <c r="D291" t="s">
+      <c r="D297" t="s">
         <v>119</v>
       </c>
-      <c r="E291" t="s">
+      <c r="E297" t="s">
         <v>120</v>
       </c>
-      <c r="F291" t="s">
+      <c r="F297" t="s">
         <v>121</v>
       </c>
-      <c r="G291" t="s">
+      <c r="G297" t="s">
         <v>122</v>
       </c>
-      <c r="H291" t="s">
+      <c r="H297" t="s">
         <v>245</v>
       </c>
-      <c r="I291" t="s">
-        <v>5</v>
-      </c>
-      <c r="J291" s="4" t="s">
+      <c r="I297" t="s">
+        <v>5</v>
+      </c>
+      <c r="J297" s="4" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B292">
+    <row r="298" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B298">
         <v>0</v>
       </c>
-      <c r="C292">
+      <c r="C298">
         <v>0.4</v>
       </c>
-      <c r="D292">
+      <c r="D298">
         <v>0.6</v>
       </c>
-      <c r="E292">
+      <c r="E298">
         <v>0</v>
       </c>
-      <c r="F292">
+      <c r="F298">
         <v>2</v>
       </c>
-      <c r="G292">
+      <c r="G298">
         <v>0.2</v>
       </c>
-      <c r="H292" s="16">
+      <c r="H298" s="16">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B293">
+    <row r="299" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B299">
         <v>0.1</v>
       </c>
-      <c r="C293">
+      <c r="C299">
         <v>0.4</v>
       </c>
-      <c r="D293">
+      <c r="D299">
         <v>0.6</v>
       </c>
-      <c r="E293">
+      <c r="E299">
         <v>0</v>
       </c>
-      <c r="F293">
+      <c r="F299">
         <v>2</v>
       </c>
-      <c r="G293">
+      <c r="G299">
         <v>0.2</v>
       </c>
-      <c r="H293" s="16">
+      <c r="H299" s="16">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B294">
-        <v>5</v>
-      </c>
-      <c r="C294">
+    <row r="300" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B300">
+        <v>5</v>
+      </c>
+      <c r="C300">
         <v>0.03</v>
       </c>
-      <c r="D294">
+      <c r="D300">
         <v>0.97</v>
       </c>
-      <c r="E294">
+      <c r="E300">
         <v>0</v>
       </c>
-      <c r="F294">
-        <v>1</v>
-      </c>
-      <c r="G294">
+      <c r="F300">
+        <v>1</v>
+      </c>
+      <c r="G300">
         <v>0.03</v>
       </c>
-      <c r="H294" s="16">
+      <c r="H300" s="16">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B295" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A296" t="s">
+    <row r="301" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B301" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="302" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A302" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A299" t="s">
+    <row r="305" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A305" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A300" t="s">
+    <row r="306" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A306" t="s">
         <v>123</v>
       </c>
-      <c r="B300" t="s">
+      <c r="B306" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A301" t="s">
+    <row r="307" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A307" t="s">
         <v>124</v>
       </c>
-      <c r="B301">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="302" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A302" s="3"/>
-      <c r="B302" s="3"/>
-      <c r="C302" t="s">
+      <c r="B307">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="308" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A308" s="3"/>
+      <c r="B308" s="3"/>
+      <c r="C308" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="303" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A303" s="7" t="s">
+    <row r="309" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A309" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B303" s="7">
+      <c r="B309" s="7">
         <v>0.25</v>
       </c>
-      <c r="C303">
+      <c r="C309">
         <v>0.2</v>
       </c>
-      <c r="D303" s="4" t="s">
+      <c r="D309" s="4" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="304" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A304" s="3" t="s">
+    <row r="310" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A310" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B304" s="3">
+      <c r="B310" s="3">
         <v>0.99</v>
       </c>
-      <c r="C304">
+      <c r="C310">
         <v>0.99</v>
       </c>
-      <c r="D304" s="4" t="s">
+      <c r="D310" s="4" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="305" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A305" s="13" t="s">
+    <row r="311" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A311" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="B305" s="13">
+      <c r="B311" s="13">
         <v>0.27</v>
       </c>
-      <c r="C305">
+      <c r="C311">
         <v>0.01</v>
       </c>
-      <c r="D305" s="4" t="s">
+      <c r="D311" s="4" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="306" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A306" s="3" t="s">
+    <row r="312" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A312" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B306" s="3">
+      <c r="B312" s="3">
         <v>0.1</v>
       </c>
-      <c r="C306">
+      <c r="C312">
         <v>0.1</v>
       </c>
-      <c r="D306" s="4" t="s">
+      <c r="D312" s="4" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="307" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A307" s="3" t="s">
+    <row r="313" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A313" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B307" s="3">
+      <c r="B313" s="3">
         <v>0.1</v>
       </c>
-      <c r="C307">
+      <c r="C313">
         <v>0.1</v>
       </c>
-      <c r="D307" s="4" t="s">
+      <c r="D313" s="4" t="s">
         <v>242</v>
-      </c>
-    </row>
-    <row r="308" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A308" t="s">
-        <v>133</v>
-      </c>
-      <c r="B308">
-        <v>0.5</v>
-      </c>
-      <c r="C308">
-        <v>0.5</v>
-      </c>
-      <c r="D308" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="309" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A309" t="s">
-        <v>135</v>
-      </c>
-      <c r="B309">
-        <v>1.0000000000000001E-5</v>
-      </c>
-      <c r="C309">
-        <v>1.0000000000000001E-5</v>
-      </c>
-      <c r="D309" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="310" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A310" t="s">
-        <v>137</v>
-      </c>
-      <c r="B310" t="s">
-        <v>138</v>
-      </c>
-      <c r="C310" t="s">
-        <v>138</v>
-      </c>
-      <c r="D310" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="311" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A311" t="s">
-        <v>140</v>
-      </c>
-      <c r="B311">
-        <v>3600</v>
-      </c>
-      <c r="C311">
-        <v>3600</v>
-      </c>
-      <c r="D311" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="312" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A312" t="s">
-        <v>142</v>
-      </c>
-      <c r="B312">
-        <v>50000</v>
-      </c>
-      <c r="C312">
-        <v>50000</v>
-      </c>
-      <c r="D312" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="313" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A313" t="s">
-        <v>144</v>
-      </c>
-      <c r="B313">
-        <v>1000</v>
-      </c>
-      <c r="C313">
-        <v>1000</v>
-      </c>
-      <c r="D313" s="4" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="B314">
-        <v>1000</v>
+        <v>0.5</v>
       </c>
       <c r="C314">
-        <v>1000</v>
+        <v>0.5</v>
       </c>
       <c r="D314" s="4" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="B315">
-        <v>-40</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="C315">
-        <v>-50</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="D315" s="4" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
-        <v>150</v>
-      </c>
-      <c r="B316">
-        <v>0.05</v>
-      </c>
-      <c r="C316">
-        <v>0.05</v>
+        <v>137</v>
+      </c>
+      <c r="B316" t="s">
+        <v>138</v>
+      </c>
+      <c r="C316" t="s">
+        <v>138</v>
       </c>
       <c r="D316" s="4" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="B317">
-        <v>0.97</v>
+        <v>3600</v>
       </c>
       <c r="C317">
-        <v>0.97</v>
+        <v>3600</v>
       </c>
       <c r="D317" s="4" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="B318">
-        <v>0.03</v>
+        <v>50000</v>
       </c>
       <c r="C318">
-        <v>0.03</v>
+        <v>50000</v>
       </c>
       <c r="D318" s="4" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
-        <v>8</v>
+        <v>144</v>
+      </c>
+      <c r="B319">
+        <v>1000</v>
+      </c>
+      <c r="C319">
+        <v>1000</v>
+      </c>
+      <c r="D319" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="320" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A320" t="s">
+        <v>146</v>
+      </c>
+      <c r="B320">
+        <v>1000</v>
+      </c>
+      <c r="C320">
+        <v>1000</v>
+      </c>
+      <c r="D320" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="321" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A321" t="s">
+        <v>148</v>
+      </c>
+      <c r="B321">
+        <v>-40</v>
+      </c>
+      <c r="C321">
+        <v>-50</v>
+      </c>
+      <c r="D321" s="4" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
-        <v>0</v>
+        <v>150</v>
+      </c>
+      <c r="B322">
+        <v>0.05</v>
+      </c>
+      <c r="C322">
+        <v>0.05</v>
+      </c>
+      <c r="D322" s="4" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
-        <v>123</v>
-      </c>
-      <c r="B323" t="s">
-        <v>2</v>
+        <v>152</v>
+      </c>
+      <c r="B323">
+        <v>0.97</v>
+      </c>
+      <c r="C323">
+        <v>0.97</v>
+      </c>
+      <c r="D323" s="4" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B324">
-        <v>1</v>
+        <v>0.03</v>
+      </c>
+      <c r="C324">
+        <v>0.03</v>
+      </c>
+      <c r="D324" s="4" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C325" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="326" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A326" t="s">
-        <v>125</v>
-      </c>
-      <c r="B326" s="5">
-        <v>0.25</v>
-      </c>
-      <c r="C326">
-        <v>0.2</v>
-      </c>
-      <c r="D326" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="327" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A327" t="s">
-        <v>127</v>
-      </c>
-      <c r="B327">
-        <v>0.99</v>
-      </c>
-      <c r="C327">
-        <v>0.99</v>
-      </c>
-      <c r="D327" s="4" t="s">
-        <v>128</v>
+      <c r="A325" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
-        <v>129</v>
-      </c>
-      <c r="B328" s="13">
-        <v>0.27</v>
-      </c>
-      <c r="C328">
-        <v>0.01</v>
-      </c>
-      <c r="D328" s="4" t="s">
-        <v>130</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
-        <v>157</v>
-      </c>
-      <c r="B329">
-        <v>0</v>
-      </c>
-      <c r="C329">
-        <v>0</v>
-      </c>
-      <c r="D329" s="4" t="s">
-        <v>158</v>
+        <v>123</v>
+      </c>
+      <c r="B329" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
-        <v>137</v>
-      </c>
-      <c r="B330" t="s">
-        <v>138</v>
-      </c>
-      <c r="C330" t="s">
-        <v>138</v>
-      </c>
-      <c r="D330" s="4" t="s">
-        <v>139</v>
+        <v>156</v>
+      </c>
+      <c r="B330">
+        <v>1</v>
       </c>
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A331" t="s">
-        <v>140</v>
-      </c>
-      <c r="B331">
-        <v>3600</v>
-      </c>
-      <c r="C331">
-        <v>3600</v>
-      </c>
-      <c r="D331" s="4" t="s">
-        <v>141</v>
+      <c r="C331" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
-        <v>142</v>
-      </c>
-      <c r="B332">
-        <v>50000</v>
+        <v>125</v>
+      </c>
+      <c r="B332" s="5">
+        <v>0.25</v>
       </c>
       <c r="C332">
-        <v>50000</v>
+        <v>0.2</v>
       </c>
       <c r="D332" s="4" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
-        <v>8</v>
+        <v>127</v>
+      </c>
+      <c r="B333">
+        <v>0.99</v>
+      </c>
+      <c r="C333">
+        <v>0.99</v>
+      </c>
+      <c r="D333" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="334" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A334" t="s">
+        <v>129</v>
+      </c>
+      <c r="B334" s="13">
+        <v>0.27</v>
+      </c>
+      <c r="C334">
+        <v>0.01</v>
+      </c>
+      <c r="D334" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="335" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A335" t="s">
+        <v>157</v>
+      </c>
+      <c r="B335">
+        <v>0</v>
+      </c>
+      <c r="C335">
+        <v>0</v>
+      </c>
+      <c r="D335" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
-        <v>0</v>
+        <v>137</v>
+      </c>
+      <c r="B336" t="s">
+        <v>138</v>
+      </c>
+      <c r="C336" t="s">
+        <v>138</v>
+      </c>
+      <c r="D336" s="4" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
-        <v>159</v>
-      </c>
-      <c r="B337" t="s">
-        <v>2</v>
+        <v>140</v>
+      </c>
+      <c r="B337">
+        <v>3600</v>
+      </c>
+      <c r="C337">
+        <v>3600</v>
+      </c>
+      <c r="D337" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
-        <v>196</v>
+        <v>142</v>
       </c>
       <c r="B338">
-        <v>1</v>
+        <v>50000</v>
+      </c>
+      <c r="C338">
+        <v>50000</v>
+      </c>
+      <c r="D338" s="4" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C339" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="340" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A340" t="s">
-        <v>197</v>
-      </c>
-      <c r="B340">
-        <v>0.85</v>
-      </c>
-      <c r="C340">
-        <v>0.85</v>
-      </c>
-      <c r="D340" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="341" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A341" t="s">
-        <v>199</v>
-      </c>
-      <c r="B341">
-        <v>0.5</v>
-      </c>
-      <c r="C341">
-        <v>0.5</v>
-      </c>
-      <c r="D341" s="4" t="s">
-        <v>200</v>
+      <c r="A339" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
-        <v>201</v>
-      </c>
-      <c r="B342">
-        <v>86400</v>
-      </c>
-      <c r="C342">
-        <v>86400</v>
-      </c>
-      <c r="D342" s="4" t="s">
-        <v>202</v>
+        <v>0</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
-        <v>203</v>
-      </c>
-      <c r="B343">
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="C343">
-        <v>8.0000000000000002E-3</v>
+        <v>159</v>
+      </c>
+      <c r="B343" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B344">
-        <v>0.24</v>
-      </c>
-      <c r="C344">
-        <v>0.24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A345" t="s">
-        <v>127</v>
-      </c>
-      <c r="B345">
-        <v>0.99</v>
-      </c>
-      <c r="C345">
-        <v>0.99</v>
-      </c>
-      <c r="D345" s="4" t="s">
-        <v>128</v>
+      <c r="C345" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
-        <v>129</v>
+        <v>197</v>
       </c>
       <c r="B346">
-        <v>0.01</v>
+        <v>0.85</v>
       </c>
       <c r="C346">
-        <v>0.01</v>
+        <v>0.85</v>
       </c>
       <c r="D346" s="4" t="s">
-        <v>130</v>
+        <v>198</v>
       </c>
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B347">
-        <v>350</v>
+        <v>0.5</v>
       </c>
       <c r="C347">
-        <v>350</v>
+        <v>0.5</v>
       </c>
       <c r="D347" s="4" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
-        <v>122</v>
+        <v>201</v>
       </c>
       <c r="B348">
-        <v>0.05</v>
+        <v>86400</v>
       </c>
       <c r="C348">
-        <v>0.05</v>
+        <v>86400</v>
       </c>
       <c r="D348" s="4" t="s">
-        <v>167</v>
+        <v>202</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
-        <v>135</v>
+        <v>203</v>
       </c>
       <c r="B349">
-        <v>1E-4</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="C349">
-        <v>1E-4</v>
-      </c>
-      <c r="D349" s="4" t="s">
-        <v>168</v>
+        <v>8.0000000000000002E-3</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
-        <v>169</v>
+        <v>204</v>
       </c>
       <c r="B350">
-        <v>0.02</v>
+        <v>0.24</v>
       </c>
       <c r="C350">
-        <v>0.02</v>
-      </c>
-      <c r="D350" s="4" t="s">
-        <v>170</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="B351">
-        <v>3600</v>
+        <v>0.99</v>
       </c>
       <c r="C351">
-        <v>3600</v>
+        <v>0.99</v>
       </c>
       <c r="D351" s="4" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="B352">
-        <v>50000</v>
+        <v>0.01</v>
       </c>
       <c r="C352">
-        <v>50000</v>
+        <v>0.01</v>
       </c>
       <c r="D352" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
-        <v>8</v>
+        <v>205</v>
+      </c>
+      <c r="B353">
+        <v>350</v>
+      </c>
+      <c r="C353">
+        <v>350</v>
+      </c>
+      <c r="D353" s="4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="354" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A354" t="s">
+        <v>122</v>
+      </c>
+      <c r="B354">
+        <v>0.05</v>
+      </c>
+      <c r="C354">
+        <v>0.05</v>
+      </c>
+      <c r="D354" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="355" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A355" t="s">
+        <v>135</v>
+      </c>
+      <c r="B355">
+        <v>1E-4</v>
+      </c>
+      <c r="C355">
+        <v>1E-4</v>
+      </c>
+      <c r="D355" s="4" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
-        <v>0</v>
+        <v>169</v>
+      </c>
+      <c r="B356">
+        <v>0.02</v>
+      </c>
+      <c r="C356">
+        <v>0.02</v>
+      </c>
+      <c r="D356" s="4" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
-        <v>159</v>
-      </c>
-      <c r="B357" t="s">
-        <v>2</v>
+        <v>140</v>
+      </c>
+      <c r="B357">
+        <v>3600</v>
+      </c>
+      <c r="C357">
+        <v>3600</v>
+      </c>
+      <c r="D357" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="B358">
-        <v>1</v>
+        <v>50000</v>
+      </c>
+      <c r="C358">
+        <v>50000</v>
+      </c>
+      <c r="D358" s="4" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C359" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="360" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A360" t="s">
-        <v>127</v>
-      </c>
-      <c r="B360">
-        <v>0.99</v>
-      </c>
-      <c r="C360">
-        <v>0.99</v>
-      </c>
-      <c r="D360" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="361" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A361" t="s">
-        <v>129</v>
-      </c>
-      <c r="B361">
-        <v>1E-3</v>
-      </c>
-      <c r="C361">
-        <v>0.01</v>
-      </c>
-      <c r="D361" s="4" t="s">
-        <v>130</v>
+      <c r="A359" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
-        <v>161</v>
-      </c>
-      <c r="B362">
-        <v>0.71</v>
-      </c>
-      <c r="C362">
-        <v>0.71</v>
-      </c>
-      <c r="D362" s="4" t="s">
-        <v>162</v>
+        <v>0</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
-        <v>163</v>
-      </c>
-      <c r="B363">
-        <v>0.21</v>
-      </c>
-      <c r="C363">
-        <v>0.21</v>
-      </c>
-      <c r="D363" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
+      </c>
+      <c r="B363" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
-        <v>165</v>
-      </c>
-      <c r="D364" s="4" t="s">
-        <v>166</v>
+        <v>160</v>
+      </c>
+      <c r="B364">
+        <v>1</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A365" t="s">
-        <v>122</v>
-      </c>
-      <c r="B365">
-        <v>0.05</v>
-      </c>
-      <c r="C365">
-        <v>0.05</v>
-      </c>
-      <c r="D365" s="4" t="s">
-        <v>167</v>
+      <c r="C365" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="B366">
-        <v>1E-4</v>
+        <v>0.99</v>
       </c>
       <c r="C366">
-        <v>1E-4</v>
+        <v>0.99</v>
       </c>
       <c r="D366" s="4" t="s">
-        <v>168</v>
+        <v>128</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
-        <v>169</v>
+        <v>129</v>
       </c>
       <c r="B367">
+        <v>1E-3</v>
+      </c>
+      <c r="C367">
         <v>0.01</v>
       </c>
-      <c r="C367">
-        <v>0.02</v>
-      </c>
       <c r="D367" s="4" t="s">
-        <v>170</v>
+        <v>130</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="B368">
-        <v>0</v>
+        <v>0.71</v>
       </c>
       <c r="C368">
-        <v>0</v>
+        <v>0.71</v>
       </c>
       <c r="D368" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
+        <v>163</v>
+      </c>
+      <c r="B369">
+        <v>0.21</v>
+      </c>
+      <c r="C369">
+        <v>0.21</v>
+      </c>
+      <c r="D369" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="370" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A370" t="s">
+        <v>165</v>
+      </c>
+      <c r="D370" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="371" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A371" t="s">
+        <v>122</v>
+      </c>
+      <c r="B371">
+        <v>0.05</v>
+      </c>
+      <c r="C371">
+        <v>0.05</v>
+      </c>
+      <c r="D371" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="372" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A372" t="s">
+        <v>135</v>
+      </c>
+      <c r="B372">
+        <v>1E-4</v>
+      </c>
+      <c r="C372">
+        <v>1E-4</v>
+      </c>
+      <c r="D372" s="4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="373" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A373" t="s">
+        <v>169</v>
+      </c>
+      <c r="B373">
+        <v>0.01</v>
+      </c>
+      <c r="C373">
+        <v>0.02</v>
+      </c>
+      <c r="D373" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="374" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A374" t="s">
+        <v>171</v>
+      </c>
+      <c r="B374">
+        <v>0</v>
+      </c>
+      <c r="C374">
+        <v>0</v>
+      </c>
+      <c r="D374" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="375" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A375" t="s">
         <v>173</v>
       </c>
-      <c r="B369">
+      <c r="B375">
         <f>48/3</f>
         <v>16</v>
       </c>
-      <c r="C369">
+      <c r="C375">
         <v>48</v>
       </c>
-      <c r="D369" s="4" t="s">
+      <c r="D375" s="4" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="370" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A370" t="s">
+    <row r="376" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A376" t="s">
         <v>175</v>
       </c>
-      <c r="B370">
+      <c r="B376">
         <v>600</v>
       </c>
-      <c r="C370">
+      <c r="C376">
         <v>350</v>
       </c>
-      <c r="D370" s="4" t="s">
+      <c r="D376" s="4" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="371" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A371" t="s">
+    <row r="377" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A377" t="s">
         <v>177</v>
       </c>
-      <c r="B371">
+      <c r="B377">
         <v>52</v>
       </c>
-      <c r="C371">
+      <c r="C377">
         <v>26</v>
       </c>
-      <c r="D371" s="4" t="s">
+      <c r="D377" s="4" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="372" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A372" t="s">
+    <row r="378" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A378" t="s">
         <v>208</v>
       </c>
-      <c r="B372">
+      <c r="B378">
         <f>0.06/60</f>
         <v>1E-3</v>
       </c>
-      <c r="D372" s="4" t="s">
+      <c r="D378" s="4" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="373" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A373" t="s">
+    <row r="379" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A379" t="s">
         <v>137</v>
       </c>
-      <c r="B373" t="s">
+      <c r="B379" t="s">
         <v>179</v>
       </c>
-      <c r="C373" t="s">
+      <c r="C379" t="s">
         <v>207</v>
       </c>
-      <c r="D373" s="4" t="s">
+      <c r="D379" s="4" t="s">
         <v>139</v>
-      </c>
-    </row>
-    <row r="374" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A374" t="s">
-        <v>140</v>
-      </c>
-      <c r="B374">
-        <v>3600</v>
-      </c>
-      <c r="C374">
-        <v>3600</v>
-      </c>
-      <c r="D374" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="375" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A375" t="s">
-        <v>142</v>
-      </c>
-      <c r="B375">
-        <v>50000</v>
-      </c>
-      <c r="C375">
-        <v>50000</v>
-      </c>
-      <c r="D375" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="376" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A376" t="s">
-        <v>239</v>
-      </c>
-      <c r="D376" s="4"/>
-    </row>
-    <row r="377" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A377" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
-        <v>0</v>
+        <v>140</v>
+      </c>
+      <c r="B380">
+        <v>3600</v>
+      </c>
+      <c r="C380">
+        <v>3600</v>
+      </c>
+      <c r="D380" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
-        <v>180</v>
-      </c>
-      <c r="B381" t="s">
-        <v>2</v>
+        <v>142</v>
+      </c>
+      <c r="B381">
+        <v>50000</v>
+      </c>
+      <c r="C381">
+        <v>50000</v>
+      </c>
+      <c r="D381" s="4" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
-        <v>34</v>
-      </c>
-      <c r="B382">
-        <v>1</v>
-      </c>
-      <c r="D382" s="4" t="s">
-        <v>244</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="D382" s="4"/>
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C383" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="384" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A384" t="s">
-        <v>181</v>
-      </c>
-      <c r="B384">
-        <v>0.25</v>
-      </c>
-      <c r="C384">
-        <v>0.25</v>
-      </c>
-      <c r="D384" s="4" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="385" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A385" t="s">
+      <c r="A383" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="386" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A386" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A387" t="s">
+        <v>180</v>
+      </c>
+      <c r="B387" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
-        <v>0</v>
+        <v>34</v>
+      </c>
+      <c r="B388">
+        <v>1</v>
+      </c>
+      <c r="D388" s="4" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A389" t="s">
-        <v>183</v>
-      </c>
-      <c r="B389" t="s">
-        <v>2</v>
+      <c r="C389" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B390">
-        <v>1</v>
+        <v>0.25</v>
+      </c>
+      <c r="C390">
+        <v>0.25</v>
+      </c>
+      <c r="D390" s="4" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C391" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="392" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A392" t="s">
-        <v>185</v>
-      </c>
-      <c r="B392">
-        <v>20</v>
-      </c>
-      <c r="C392">
-        <v>10000</v>
-      </c>
-      <c r="D392" s="4" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="393" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A393" t="s">
-        <v>187</v>
-      </c>
-      <c r="B393">
-        <v>0</v>
-      </c>
-      <c r="C393">
-        <v>0</v>
-      </c>
-      <c r="D393" s="4" t="s">
-        <v>188</v>
+      <c r="A391" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
-        <v>189</v>
-      </c>
-      <c r="B394">
-        <v>0.03</v>
-      </c>
-      <c r="C394">
-        <v>0.03</v>
-      </c>
-      <c r="D394" s="4" t="s">
-        <v>190</v>
+        <v>0</v>
       </c>
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
-        <v>191</v>
-      </c>
-      <c r="B395">
-        <v>5</v>
-      </c>
-      <c r="C395">
-        <v>1</v>
-      </c>
-      <c r="D395" s="4" t="s">
-        <v>192</v>
+        <v>183</v>
+      </c>
+      <c r="B395" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B396">
         <v>1</v>
       </c>
-      <c r="C396">
-        <v>1</v>
-      </c>
-      <c r="D396" s="4" t="s">
-        <v>194</v>
-      </c>
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A397" t="s">
-        <v>8</v>
+      <c r="C397" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="398" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A398" t="s">
+        <v>185</v>
+      </c>
+      <c r="B398">
+        <v>20</v>
+      </c>
+      <c r="C398">
+        <v>10000</v>
+      </c>
+      <c r="D398" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="399" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A399" t="s">
+        <v>187</v>
+      </c>
+      <c r="B399">
+        <v>0</v>
+      </c>
+      <c r="C399">
+        <v>0</v>
+      </c>
+      <c r="D399" s="4" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
+        <v>189</v>
+      </c>
+      <c r="B400">
+        <v>0.03</v>
+      </c>
+      <c r="C400">
+        <v>0.03</v>
+      </c>
+      <c r="D400" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="401" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A401" t="s">
+        <v>191</v>
+      </c>
+      <c r="B401">
+        <v>5</v>
+      </c>
+      <c r="C401">
+        <v>1</v>
+      </c>
+      <c r="D401" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="402" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A402" t="s">
+        <v>193</v>
+      </c>
+      <c r="B402">
+        <v>1</v>
+      </c>
+      <c r="C402">
+        <v>1</v>
+      </c>
+      <c r="D402" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="403" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A403" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="406" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A406" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="401" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A401" t="s">
+    <row r="407" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A407" t="s">
         <v>183</v>
       </c>
-      <c r="B401" t="s">
+      <c r="B407" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="402" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A402" t="s">
+    <row r="408" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A408" t="s">
         <v>195</v>
       </c>
-      <c r="B402">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="404" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A404" t="s">
+      <c r="B408">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="410" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A410" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>